<commit_message>
docs: Correct variable explanations in codebook
</commit_message>
<xml_diff>
--- a/data/feature_target_explanations.xlsx
+++ b/data/feature_target_explanations.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charles.plumridge\Documents\VSCode\portfolio\foreign-student-mental-health-ml\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A898BE73-6090-4227-AA36-4A173F689240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D5C414-F328-42D1-9A44-67528ABBA5A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="17520" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cat_variables" sheetId="1" r:id="rId1"/>
     <sheet name="numeric_variables" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -280,9 +279,6 @@
     <t>ToAS</t>
   </si>
   <si>
-    <t>Total score of Acculturative Stress</t>
-  </si>
-  <si>
     <t>Partner</t>
   </si>
   <si>
@@ -416,6 +412,9 @@
   </si>
   <si>
     <t>Self-evaluation scale ranging from 1 to 5 regarding English proficiency: High (4 to 5), Average (3) or Low (1 to 2)</t>
+  </si>
+  <si>
+    <t>Total score of Acculturative Stress measured by ASISS questionnaire</t>
   </si>
 </sst>
 </file>
@@ -892,44 +891,44 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" style="1" customWidth="1"/>
-    <col min="3" max="5" width="11.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="82.109375" customWidth="1"/>
-    <col min="7" max="7" width="33.109375" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" style="1" customWidth="1"/>
+    <col min="3" max="5" width="11.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="82.140625" customWidth="1"/>
+    <col min="7" max="7" width="33.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C2" s="5">
         <v>3</v>
@@ -944,15 +943,15 @@
         <v>4</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C3" s="7">
         <v>1</v>
@@ -964,18 +963,18 @@
         <v>2</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C4" s="5">
         <v>3</v>
@@ -990,15 +989,15 @@
         <v>8</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C5" s="7">
         <v>3</v>
@@ -1013,15 +1012,15 @@
         <v>10</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C6" s="5">
         <v>3</v>
@@ -1033,18 +1032,18 @@
         <v>1</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C7" s="7">
         <v>3</v>
@@ -1059,15 +1058,15 @@
         <v>12</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C8" s="5">
         <v>3</v>
@@ -1079,18 +1078,18 @@
         <v>2</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C9" s="7">
         <v>3</v>
@@ -1102,18 +1101,18 @@
         <v>2</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C10" s="5">
         <v>3</v>
@@ -1128,15 +1127,15 @@
         <v>16</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>17</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C11" s="7">
         <v>3</v>
@@ -1151,15 +1150,15 @@
         <v>18</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C12" s="5">
         <v>0</v>
@@ -1174,15 +1173,15 @@
         <v>20</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C13" s="7">
         <v>0</v>
@@ -1197,15 +1196,15 @@
         <v>22</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C14" s="5">
         <v>0</v>
@@ -1220,15 +1219,15 @@
         <v>24</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>25</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C15" s="7">
         <v>0</v>
@@ -1243,15 +1242,15 @@
         <v>26</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>28</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C16" s="5">
         <v>1</v>
@@ -1266,15 +1265,15 @@
         <v>29</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C17" s="7">
         <v>1</v>
@@ -1289,15 +1288,15 @@
         <v>31</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C18" s="5">
         <v>1</v>
@@ -1312,15 +1311,15 @@
         <v>33</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>34</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C19" s="7">
         <v>1</v>
@@ -1335,15 +1334,15 @@
         <v>35</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>36</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C20" s="5">
         <v>1</v>
@@ -1358,15 +1357,15 @@
         <v>37</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>38</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C21" s="7">
         <v>1</v>
@@ -1381,15 +1380,15 @@
         <v>39</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>40</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C22" s="5">
         <v>1</v>
@@ -1404,15 +1403,15 @@
         <v>41</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>42</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C23" s="7">
         <v>1</v>
@@ -1427,15 +1426,15 @@
         <v>43</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>44</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C24" s="5">
         <v>1</v>
@@ -1450,15 +1449,15 @@
         <v>45</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>46</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C25" s="7">
         <v>1</v>
@@ -1473,15 +1472,15 @@
         <v>47</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>48</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C26" s="5">
         <v>1</v>
@@ -1496,7 +1495,7 @@
         <v>49</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1522,26 +1521,26 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBE1E3CB-FA04-4921-AB37-FFB1E5A0A5D0}">
   <dimension ref="A1:J26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5546875" customWidth="1"/>
-    <col min="2" max="4" width="11.33203125" customWidth="1"/>
-    <col min="5" max="5" width="66.44140625" customWidth="1"/>
-    <col min="6" max="10" width="10.5546875" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+    <col min="2" max="4" width="11.28515625" customWidth="1"/>
+    <col min="5" max="5" width="66.42578125" customWidth="1"/>
+    <col min="6" max="10" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>114</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>115</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>1</v>
@@ -1562,7 +1561,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>53</v>
       </c>
@@ -1594,7 +1593,7 @@
         <v>2.77</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>55</v>
       </c>
@@ -1626,9 +1625,9 @@
         <v>1.33</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B4" s="9">
         <v>3</v>
@@ -1658,9 +1657,9 @@
         <v>1.31</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B5" s="7">
         <v>3</v>
@@ -1690,7 +1689,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>61</v>
       </c>
@@ -1722,7 +1721,7 @@
         <v>4.95</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>63</v>
       </c>
@@ -1754,7 +1753,7 @@
         <v>9.23</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>65</v>
       </c>
@@ -1786,7 +1785,7 @@
         <v>6.17</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>67</v>
       </c>
@@ -1818,7 +1817,7 @@
         <v>4.01</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>69</v>
       </c>
@@ -1850,7 +1849,7 @@
         <v>4.1900000000000004</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>71</v>
       </c>
@@ -1882,7 +1881,7 @@
         <v>3.11</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>73</v>
       </c>
@@ -1914,7 +1913,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>75</v>
       </c>
@@ -1946,7 +1945,7 @@
         <v>1.91</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>77</v>
       </c>
@@ -1978,7 +1977,7 @@
         <v>7.4</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>79</v>
       </c>
@@ -1992,7 +1991,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>80</v>
+        <v>125</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>59</v>
@@ -2010,21 +2009,21 @@
         <v>22.64</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" s="9">
+        <v>1</v>
+      </c>
+      <c r="C16" s="9">
+        <v>1</v>
+      </c>
+      <c r="D16" s="9">
+        <v>1</v>
+      </c>
+      <c r="E16" s="8" t="s">
         <v>81</v>
-      </c>
-      <c r="B16" s="9">
-        <v>1</v>
-      </c>
-      <c r="C16" s="9">
-        <v>1</v>
-      </c>
-      <c r="D16" s="9">
-        <v>1</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>82</v>
       </c>
       <c r="F16" s="10" t="s">
         <v>59</v>
@@ -2042,21 +2041,21 @@
         <v>2.23</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="7">
+        <v>1</v>
+      </c>
+      <c r="C17" s="7">
+        <v>1</v>
+      </c>
+      <c r="D17" s="7">
+        <v>1</v>
+      </c>
+      <c r="E17" s="11" t="s">
         <v>83</v>
-      </c>
-      <c r="B17" s="7">
-        <v>1</v>
-      </c>
-      <c r="C17" s="7">
-        <v>1</v>
-      </c>
-      <c r="D17" s="7">
-        <v>1</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>84</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>59</v>
@@ -2074,21 +2073,21 @@
         <v>1.94</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B18" s="9">
+        <v>1</v>
+      </c>
+      <c r="C18" s="9">
+        <v>1</v>
+      </c>
+      <c r="D18" s="9">
+        <v>1</v>
+      </c>
+      <c r="E18" s="8" t="s">
         <v>85</v>
-      </c>
-      <c r="B18" s="9">
-        <v>1</v>
-      </c>
-      <c r="C18" s="9">
-        <v>1</v>
-      </c>
-      <c r="D18" s="9">
-        <v>1</v>
-      </c>
-      <c r="E18" s="8" t="s">
-        <v>86</v>
       </c>
       <c r="F18" s="10" t="s">
         <v>59</v>
@@ -2106,21 +2105,21 @@
         <v>2.0699999999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="7">
+        <v>1</v>
+      </c>
+      <c r="C19" s="7">
+        <v>1</v>
+      </c>
+      <c r="D19" s="7">
+        <v>1</v>
+      </c>
+      <c r="E19" s="11" t="s">
         <v>87</v>
-      </c>
-      <c r="B19" s="7">
-        <v>1</v>
-      </c>
-      <c r="C19" s="7">
-        <v>1</v>
-      </c>
-      <c r="D19" s="7">
-        <v>1</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>88</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>59</v>
@@ -2138,21 +2137,21 @@
         <v>1.85</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" s="9">
+        <v>1</v>
+      </c>
+      <c r="C20" s="9">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9">
+        <v>1</v>
+      </c>
+      <c r="E20" s="8" t="s">
         <v>89</v>
-      </c>
-      <c r="B20" s="9">
-        <v>1</v>
-      </c>
-      <c r="C20" s="9">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9">
-        <v>1</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>90</v>
       </c>
       <c r="F20" s="10" t="s">
         <v>59</v>
@@ -2170,21 +2169,21 @@
         <v>1.83</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B21" s="7">
+        <v>1</v>
+      </c>
+      <c r="C21" s="7">
+        <v>1</v>
+      </c>
+      <c r="D21" s="7">
+        <v>1</v>
+      </c>
+      <c r="E21" s="11" t="s">
         <v>91</v>
-      </c>
-      <c r="B21" s="7">
-        <v>1</v>
-      </c>
-      <c r="C21" s="7">
-        <v>1</v>
-      </c>
-      <c r="D21" s="7">
-        <v>1</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>92</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>59</v>
@@ -2202,21 +2201,21 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B22" s="9">
+        <v>1</v>
+      </c>
+      <c r="C22" s="9">
+        <v>1</v>
+      </c>
+      <c r="D22" s="9">
+        <v>1</v>
+      </c>
+      <c r="E22" s="8" t="s">
         <v>93</v>
-      </c>
-      <c r="B22" s="9">
-        <v>1</v>
-      </c>
-      <c r="C22" s="9">
-        <v>1</v>
-      </c>
-      <c r="D22" s="9">
-        <v>1</v>
-      </c>
-      <c r="E22" s="8" t="s">
-        <v>94</v>
       </c>
       <c r="F22" s="10" t="s">
         <v>59</v>
@@ -2234,21 +2233,21 @@
         <v>1.71</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B23" s="7">
+        <v>1</v>
+      </c>
+      <c r="C23" s="7">
+        <v>1</v>
+      </c>
+      <c r="D23" s="7">
+        <v>1</v>
+      </c>
+      <c r="E23" s="11" t="s">
         <v>95</v>
-      </c>
-      <c r="B23" s="7">
-        <v>1</v>
-      </c>
-      <c r="C23" s="7">
-        <v>1</v>
-      </c>
-      <c r="D23" s="7">
-        <v>1</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>96</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>59</v>
@@ -2266,21 +2265,21 @@
         <v>1.41</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B24" s="9">
+        <v>1</v>
+      </c>
+      <c r="C24" s="9">
+        <v>1</v>
+      </c>
+      <c r="D24" s="9">
+        <v>1</v>
+      </c>
+      <c r="E24" s="8" t="s">
         <v>97</v>
-      </c>
-      <c r="B24" s="9">
-        <v>1</v>
-      </c>
-      <c r="C24" s="9">
-        <v>1</v>
-      </c>
-      <c r="D24" s="9">
-        <v>1</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>98</v>
       </c>
       <c r="F24" s="10" t="s">
         <v>59</v>
@@ -2298,7 +2297,7 @@
         <v>2.0299999999999998</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
         <v>6</v>
       </c>
@@ -2312,7 +2311,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>59</v>
@@ -2330,21 +2329,21 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="B26" s="9">
+        <v>1</v>
+      </c>
+      <c r="C26" s="9">
+        <v>1</v>
+      </c>
+      <c r="D26" s="9">
+        <v>1</v>
+      </c>
+      <c r="E26" s="8" t="s">
         <v>100</v>
-      </c>
-      <c r="B26" s="9">
-        <v>1</v>
-      </c>
-      <c r="C26" s="9">
-        <v>1</v>
-      </c>
-      <c r="D26" s="9">
-        <v>1</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>101</v>
       </c>
       <c r="F26" s="10" t="s">
         <v>59</v>

</xml_diff>